<commit_message>
Removed two 100 values that did not need to be there.
</commit_message>
<xml_diff>
--- a/_Exam_grade_template.xlsx
+++ b/_Exam_grade_template.xlsx
@@ -1,16 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="20910"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="28502"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/goby/Documents/teach/exams/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="15520" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="15460" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="140000" concurrentCalc="0"/>
+  <calcPr calcId="150001" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr defaultImageDpi="32767"/>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
     </ext>
@@ -236,6 +244,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -317,7 +330,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.0</c:v>
+                  <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -359,7 +372,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>2.0</c:v>
+                  <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.0</c:v>
@@ -371,7 +384,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>162.0</c:v>
+                  <c:v>164.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -386,16 +399,17 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="2074926632"/>
-        <c:axId val="2074929640"/>
+        <c:axId val="680777088"/>
+        <c:axId val="680781088"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2074926632"/>
+        <c:axId val="680777088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -409,7 +423,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2074929640"/>
+        <c:crossAx val="680781088"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -417,7 +431,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2074929640"/>
+        <c:axId val="680781088"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -437,7 +451,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2074926632"/>
+        <c:crossAx val="680777088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -841,9 +855,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H165"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -854,13 +868,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2">
-        <v>100</v>
-      </c>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B2" s="2">
         <f t="shared" ref="B2:B33" si="0">A2+$C$1</f>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>5</v>
@@ -872,30 +883,27 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3">
-        <v>100</v>
-      </c>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B3" s="1">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="5" t="e">
         <f>AVERAGE(A2:A167)</f>
-        <v>100</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F3" s="5">
         <f>AVERAGE(B2:B167)</f>
-        <v>1.2195121951219512</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B4" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -903,16 +911,16 @@
       <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="5" t="e">
         <f>_xlfn.STDEV.S(A2:A165)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F4" s="5"/>
       <c r="H4">
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -920,16 +928,16 @@
       <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="5" t="e">
         <f>E4/SQRT(F13)</f>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="F5" s="5"/>
       <c r="H5">
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B6" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -939,7 +947,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B7" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -949,14 +957,14 @@
       </c>
       <c r="E7">
         <f>COUNTIFS(A2:A165,"&gt;="&amp;$H$3)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7">
         <f>COUNTIFS(B2:B165,"&gt;="&amp;$H$3)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B8" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -973,7 +981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B9" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -990,7 +998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B10" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1007,7 +1015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B11" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1021,17 +1029,17 @@
       </c>
       <c r="F11">
         <f>COUNTIFS(B2:B165,"&lt;"&amp;$H6)</f>
-        <v>162</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B12" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B13" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1041,920 +1049,920 @@
       </c>
       <c r="E13">
         <f>SUM(E7:E11)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <f>SUM(F7:F11)</f>
         <v>164</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B14" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B15" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B16" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B19" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B20" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B21" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B22" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B23" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B24" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B25" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B26" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B27" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B28" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B29" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B30" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B31" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B32" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B33" s="1">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B34" s="1">
         <f t="shared" ref="B34:B65" si="1">A34+$C$1</f>
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B35" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B36" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B37" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B38" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B39" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B40" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B41" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B42" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B43" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B44" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B45" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B46" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B47" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B48" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B49" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B50" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B51" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B52" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B53" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B54" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B55" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B56" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B57" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B58" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B59" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B60" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B61" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B62" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B63" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B64" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B65" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B66" s="1">
         <f t="shared" ref="B66:B97" si="2">A66+$C$1</f>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B67" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B68" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B69" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B70" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B71" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B72" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B73" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B74" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B75" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B76" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B77" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B78" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B79" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B80" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B81" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B82" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B83" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B84" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B85" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B86" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B87" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B88" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B89" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B90" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B91" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B92" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B93" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B94" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B95" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B96" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B97" s="1">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B98" s="1">
         <f t="shared" ref="B98:B129" si="3">A98+$C$1</f>
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B99" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B100" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B101" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B102" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B103" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B104" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B105" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B106" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B107" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B108" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B109" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B110" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B111" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B112" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B113" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B114" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B115" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B116" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B117" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B118" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B119" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B120" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B121" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B122" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B123" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B124" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B125" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B126" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B127" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B128" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B129" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B130" s="1">
         <f t="shared" ref="B130:B161" si="4">A130+$C$1</f>
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B131" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B132" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B133" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B134" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B135" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B136" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B137" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B138" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B139" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B140" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B141" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B142" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B143" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B144" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B145" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B146" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B147" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B148" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B149" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B150" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B151" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B152" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B153" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B154" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B155" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B156" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B157" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B158" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B159" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B160" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B161" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B162" s="1">
-        <f t="shared" ref="B162:B193" si="5">A162+$C$1</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" spans="2:2">
+        <f t="shared" ref="B162:B165" si="5">A162+$C$1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B163" s="1">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B164" s="1">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B165" s="1">
         <f t="shared" si="5"/>
         <v>0</v>
@@ -1967,10 +1975,5 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <drawing r:id="rId1"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Using only first 100 rows
</commit_message>
<xml_diff>
--- a/_Exam_grade_template.xlsx
+++ b/_Exam_grade_template.xlsx
@@ -384,7 +384,7 @@
                   <c:v>0.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>164.0</c:v>
+                  <c:v>100.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -399,11 +399,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="680777088"/>
-        <c:axId val="680781088"/>
+        <c:axId val="-1297876608"/>
+        <c:axId val="-1297874288"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="680777088"/>
+        <c:axId val="-1297876608"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -423,7 +423,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="680781088"/>
+        <c:crossAx val="-1297874288"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -431,7 +431,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="680781088"/>
+        <c:axId val="-1297874288"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -451,7 +451,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="680777088"/>
+        <c:crossAx val="-1297876608"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="F11">
         <f>COUNTIFS(B2:B165,"&lt;"&amp;$H6)</f>
-        <v>164</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F13">
         <f>SUM(F7:F11)</f>
-        <v>164</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1585,388 +1585,196 @@
       </c>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B102" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B102" s="1"/>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B103" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B103" s="1"/>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B104" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B104" s="1"/>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B105" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B105" s="1"/>
     </row>
     <row r="106" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B106" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B106" s="1"/>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B107" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B107" s="1"/>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B108" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B108" s="1"/>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B109" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B109" s="1"/>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B110" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B110" s="1"/>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B111" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B111" s="1"/>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B112" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B112" s="1"/>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B113" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B113" s="1"/>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B114" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B114" s="1"/>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B115" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B115" s="1"/>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B116" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B116" s="1"/>
     </row>
     <row r="117" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B117" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B117" s="1"/>
     </row>
     <row r="118" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B118" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B118" s="1"/>
     </row>
     <row r="119" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B119" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B119" s="1"/>
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B120" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B120" s="1"/>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B121" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B121" s="1"/>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B122" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B122" s="1"/>
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B123" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B123" s="1"/>
     </row>
     <row r="124" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B124" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B124" s="1"/>
     </row>
     <row r="125" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B125" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B125" s="1"/>
     </row>
     <row r="126" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B126" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B126" s="1"/>
     </row>
     <row r="127" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B127" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B127" s="1"/>
     </row>
     <row r="128" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B128" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B128" s="1"/>
     </row>
     <row r="129" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B129" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B129" s="1"/>
     </row>
     <row r="130" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B130" s="1">
-        <f t="shared" ref="B130:B161" si="4">A130+$C$1</f>
-        <v>0</v>
-      </c>
+      <c r="B130" s="1"/>
     </row>
     <row r="131" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B131" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B131" s="1"/>
     </row>
     <row r="132" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B132" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B132" s="1"/>
     </row>
     <row r="133" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B133" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B133" s="1"/>
     </row>
     <row r="134" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B134" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B134" s="1"/>
     </row>
     <row r="135" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B135" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B135" s="1"/>
     </row>
     <row r="136" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B136" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B136" s="1"/>
     </row>
     <row r="137" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B137" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B137" s="1"/>
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B138" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B138" s="1"/>
     </row>
     <row r="139" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B139" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B139" s="1"/>
     </row>
     <row r="140" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B140" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B140" s="1"/>
     </row>
     <row r="141" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B141" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B141" s="1"/>
     </row>
     <row r="142" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B142" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B142" s="1"/>
     </row>
     <row r="143" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B143" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B143" s="1"/>
     </row>
     <row r="144" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B144" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B144" s="1"/>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B145" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B145" s="1"/>
     </row>
     <row r="146" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B146" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B146" s="1"/>
     </row>
     <row r="147" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B147" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B147" s="1"/>
     </row>
     <row r="148" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B148" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B148" s="1"/>
     </row>
     <row r="149" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B149" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B149" s="1"/>
     </row>
     <row r="150" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B150" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B150" s="1"/>
     </row>
     <row r="151" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B151" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B151" s="1"/>
     </row>
     <row r="152" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B152" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B152" s="1"/>
     </row>
     <row r="153" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B153" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B153" s="1"/>
     </row>
     <row r="154" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B154" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B154" s="1"/>
     </row>
     <row r="155" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B155" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B155" s="1"/>
     </row>
     <row r="156" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B156" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B156" s="1"/>
     </row>
     <row r="157" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B157" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B157" s="1"/>
     </row>
     <row r="158" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B158" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B158" s="1"/>
     </row>
     <row r="159" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B159" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B159" s="1"/>
     </row>
     <row r="160" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B160" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B160" s="1"/>
     </row>
     <row r="161" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B161" s="1">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="B161" s="1"/>
     </row>
     <row r="162" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B162" s="1">
-        <f t="shared" ref="B162:B165" si="5">A162+$C$1</f>
-        <v>0</v>
-      </c>
+      <c r="B162" s="1"/>
     </row>
     <row r="163" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B163" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
+      <c r="B163" s="1"/>
     </row>
     <row r="164" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B164" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
+      <c r="B164" s="1"/>
     </row>
     <row r="165" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B165" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
+      <c r="B165" s="1"/>
     </row>
   </sheetData>
   <sortState ref="A2:B165">

</xml_diff>

<commit_message>
Reduce students to 40
</commit_message>
<xml_diff>
--- a/_Exam_grade_template.xlsx
+++ b/_Exam_grade_template.xlsx
@@ -1,23 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="28502"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
   <workbookPr showInkAnnotation="0" hidePivotFieldList="1" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/goby/Documents/teach/exams/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mtaylor/Documents/teach/exams/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD857927-EE86-1B42-90D9-98317EDF225E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="15460" tabRatio="500"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="25600" windowHeight="15460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="150001" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -68,7 +80,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
@@ -248,12 +260,15 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -274,9 +289,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="0.109077615298088"/>
-          <c:y val="0.0381221088473471"/>
-          <c:w val="0.85026209223847"/>
-          <c:h val="0.86888632519797"/>
+          <c:y val="3.8122108847347097E-2"/>
+          <c:w val="0.85026209223847005"/>
+          <c:h val="0.86888632519797004"/>
         </c:manualLayout>
       </c:layout>
       <c:barChart>
@@ -330,23 +345,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-693B-C94D-A8E9-0D9E46344114}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -372,23 +392,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>100.0</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-693B-C94D-A8E9-0D9E46344114}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:dLbls>
           <c:showLegendKey val="0"/>
@@ -463,9 +488,9 @@
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
           <c:x val="0.15889457567804"/>
-          <c:y val="0.092208734324876"/>
+          <c:y val="9.2208734324876002E-2"/>
           <c:w val="0.15930461192351"/>
-          <c:h val="0.12801424715225"/>
+          <c:h val="0.12801424715224999"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -491,7 +516,7 @@
   </c:spPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="1.0" l="0.75" r="0.75" t="1.0" header="0.5" footer="0.5"/>
+    <c:pageMargins b="1" l="0.75" r="0.75" t="1" header="0.5" footer="0.5"/>
     <c:pageSetup/>
   </c:printSettings>
 </c:chartSpace>
@@ -514,7 +539,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -853,7 +884,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H165"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -892,11 +923,11 @@
         <v>7</v>
       </c>
       <c r="E3" s="5" t="e">
-        <f>AVERAGE(A2:A167)</f>
+        <f>AVERAGE(A2:A41)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F3" s="5">
-        <f>AVERAGE(B2:B167)</f>
+        <f>AVERAGE(B2:B41)</f>
         <v>0</v>
       </c>
       <c r="H3">
@@ -912,7 +943,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="5" t="e">
-        <f>_xlfn.STDEV.S(A2:A165)</f>
+        <f>_xlfn.STDEV.S(A2:A41)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="F4" s="5"/>
@@ -956,11 +987,11 @@
         <v>0</v>
       </c>
       <c r="E7">
-        <f>COUNTIFS(A2:A165,"&gt;="&amp;$H$3)</f>
+        <f>COUNTIFS(A2:A41,"&gt;="&amp;$H$3)</f>
         <v>0</v>
       </c>
       <c r="F7">
-        <f>COUNTIFS(B2:B165,"&gt;="&amp;$H$3)</f>
+        <f>COUNTIFS(B2:B41,"&gt;="&amp;$H$3)</f>
         <v>0</v>
       </c>
     </row>
@@ -973,11 +1004,11 @@
         <v>1</v>
       </c>
       <c r="E8">
-        <f>COUNTIFS(A2:A165,"&gt;="&amp;$H$4,A2:A165,"&lt;"&amp;$H$3)</f>
+        <f>COUNTIFS(A2:A41,"&gt;="&amp;$H$4,A2:A41,"&lt;"&amp;$H$3)</f>
         <v>0</v>
       </c>
       <c r="F8">
-        <f>COUNTIFS(B2:B165,"&gt;="&amp;$H$4,B2:B165,"&lt;"&amp;$H$3)</f>
+        <f>COUNTIFS(B2:B41,"&gt;="&amp;$H$4,B2:B41,"&lt;"&amp;$H$3)</f>
         <v>0</v>
       </c>
     </row>
@@ -990,11 +1021,11 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <f>COUNTIFS(A2:A165,"&gt;="&amp;$H5,A2:A165,"&lt;"&amp;$H4)</f>
+        <f>COUNTIFS(A2:A41,"&gt;="&amp;$H5,A2:A41,"&lt;"&amp;$H4)</f>
         <v>0</v>
       </c>
       <c r="F9">
-        <f>COUNTIFS(B2:B165,"&gt;="&amp;$H5,B2:B165,"&lt;"&amp;$H4)</f>
+        <f>COUNTIFS(B2:B41,"&gt;="&amp;$H5,B2:B41,"&lt;"&amp;$H4)</f>
         <v>0</v>
       </c>
     </row>
@@ -1007,11 +1038,11 @@
         <v>3</v>
       </c>
       <c r="E10">
-        <f>COUNTIFS(A2:A165,"&gt;="&amp;$H6,A2:A165,"&lt;"&amp;$H5)</f>
+        <f>COUNTIFS(A2:A41,"&gt;="&amp;$H6,A2:A41,"&lt;"&amp;$H5)</f>
         <v>0</v>
       </c>
       <c r="F10">
-        <f>COUNTIFS(B2:B165,"&gt;="&amp;$H6,B2:B165,"&lt;"&amp;$H5)</f>
+        <f>COUNTIFS(B2:B41,"&gt;="&amp;$H6,B2:B41,"&lt;"&amp;$H5)</f>
         <v>0</v>
       </c>
     </row>
@@ -1024,12 +1055,12 @@
         <v>4</v>
       </c>
       <c r="E11">
-        <f>COUNTIFS(A2:A165,"&lt;"&amp;$H6)</f>
+        <f>COUNTIFS(A2:A41,"&lt;"&amp;$H6)</f>
         <v>0</v>
       </c>
       <c r="F11">
-        <f>COUNTIFS(B2:B165,"&lt;"&amp;$H6)</f>
-        <v>100</v>
+        <f>COUNTIFS(B2:B41,"&lt;"&amp;$H6)</f>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -1053,7 +1084,7 @@
       </c>
       <c r="F13">
         <f>SUM(F7:F11)</f>
-        <v>100</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1225,364 +1256,184 @@
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B42" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B42" s="1"/>
     </row>
     <row r="43" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B43" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B43" s="1"/>
     </row>
     <row r="44" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B44" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B44" s="1"/>
     </row>
     <row r="45" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B45" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B45" s="1"/>
     </row>
     <row r="46" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B46" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B46" s="1"/>
     </row>
     <row r="47" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B47" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B47" s="1"/>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B48" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B48" s="1"/>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B49" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B49" s="1"/>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B50" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B50" s="1"/>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B51" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B51" s="1"/>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B52" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B52" s="1"/>
     </row>
     <row r="53" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B53" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B53" s="1"/>
     </row>
     <row r="54" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B54" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B54" s="1"/>
     </row>
     <row r="55" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B55" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B55" s="1"/>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B56" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B56" s="1"/>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B57" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B57" s="1"/>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B58" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B58" s="1"/>
     </row>
     <row r="59" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B59" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B59" s="1"/>
     </row>
     <row r="60" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B60" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B60" s="1"/>
     </row>
     <row r="61" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B61" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B61" s="1"/>
     </row>
     <row r="62" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B62" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B62" s="1"/>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B63" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B63" s="1"/>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B64" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B64" s="1"/>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B65" s="1">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="B65" s="1"/>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B66" s="1">
-        <f t="shared" ref="B66:B97" si="2">A66+$C$1</f>
-        <v>0</v>
-      </c>
+      <c r="B66" s="1"/>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B67" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B67" s="1"/>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B68" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B68" s="1"/>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B69" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B69" s="1"/>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B70" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B70" s="1"/>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B71" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B71" s="1"/>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B72" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B72" s="1"/>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B73" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B73" s="1"/>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B74" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B74" s="1"/>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B75" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B75" s="1"/>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B76" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B76" s="1"/>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B77" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B77" s="1"/>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B78" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B78" s="1"/>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B79" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B79" s="1"/>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B80" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B80" s="1"/>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B81" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B81" s="1"/>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B82" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B82" s="1"/>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B83" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B83" s="1"/>
     </row>
     <row r="84" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B84" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B84" s="1"/>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B85" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B85" s="1"/>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B86" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B86" s="1"/>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B87" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B87" s="1"/>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B88" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B88" s="1"/>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B89" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B89" s="1"/>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B90" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B90" s="1"/>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B91" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B91" s="1"/>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B92" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B92" s="1"/>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B93" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B93" s="1"/>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B94" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B94" s="1"/>
     </row>
     <row r="95" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B95" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B95" s="1"/>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B96" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B96" s="1"/>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B97" s="1">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="B97" s="1"/>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B98" s="1">
-        <f t="shared" ref="B98:B129" si="3">A98+$C$1</f>
-        <v>0</v>
-      </c>
+      <c r="B98" s="1"/>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B99" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B99" s="1"/>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B100" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B100" s="1"/>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B101" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="B101" s="1"/>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B102" s="1"/>
@@ -1777,7 +1628,7 @@
       <c r="B165" s="1"/>
     </row>
   </sheetData>
-  <sortState ref="A2:B165">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B165">
     <sortCondition descending="1" ref="A2:A165"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>